<commit_message>
Ajustes de la revisión: indirectos, costo unitario, MVP y animaciones
- Gastos indirectos (publicidad, 30 % de la operación) sumados al precio:
  Agente $1,56 M, MVP $3,25 M, Operación $3,9 M.
- Costo unitario (I+D) y margen de ganancia por cliente; equilibrio en 22.
- Dato de errores en la digitación manual y puestos que automatiza el agente.
- "Piloto" pasa a MVP, "PyMe" con mayúsculas y sin la etiqueta de persona
  ficticia.
- Animaciones de entrada por slide; guion y Excel actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/informe/Kiwano_red_de_nodos.xlsx
+++ b/informe/Kiwano_red_de_nodos.xlsx
@@ -923,7 +923,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>PYME de 35 años que cotiza por WhatsApp: agente cotizador y automatización de pagos y guías.</t>
+          <t>PyMe de 35 años que cotiza por WhatsApp: agente cotizador y automatización de pagos y guías.</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Outsourcing contable, tributario y legal para pymes</t>
+          <t>Outsourcing contable, tributario y legal para PyMes</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>El competidor más directo: RPA + IA para pymes, incluida logística, en la misma zona.</t>
+          <t>El competidor más directo: RPA + IA para PyMes, incluida logística, en la misma zona.</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -4532,10 +4532,10 @@
         </is>
       </c>
       <c r="D18" s="14" t="n">
-        <v>96000</v>
+        <v>124800</v>
       </c>
       <c r="E18" s="14" t="n">
-        <v>96000</v>
+        <v>124800</v>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
@@ -4560,10 +4560,10 @@
         </is>
       </c>
       <c r="D19" s="14" t="n">
-        <v>70800</v>
+        <v>92040</v>
       </c>
       <c r="E19" s="14" t="n">
-        <v>70800</v>
+        <v>92040</v>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
@@ -4588,10 +4588,10 @@
         </is>
       </c>
       <c r="D20" s="14" t="n">
-        <v>38640</v>
+        <v>50232</v>
       </c>
       <c r="E20" s="14" t="n">
-        <v>38640</v>
+        <v>50232</v>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="E25" s="16" t="n">
-        <v>1200000</v>
+        <v>1560000</v>
       </c>
     </row>
     <row r="26">
@@ -4700,7 +4700,7 @@
         </is>
       </c>
       <c r="E26" s="16" t="n">
-        <v>265440</v>
+        <v>327072</v>
       </c>
     </row>
     <row r="27">
@@ -4710,7 +4710,7 @@
         </is>
       </c>
       <c r="E27" s="16" t="n">
-        <v>934560</v>
+        <v>1232928</v>
       </c>
     </row>
     <row r="28">
@@ -4730,7 +4730,7 @@
         </is>
       </c>
       <c r="E29" s="9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -4805,11 +4805,11 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Piloto</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>2500000</v>
+        <v>3250000</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Un proceso, 6 semanas.</t>
+          <t>Un proceso funcionando en 6 semanas.</t>
         </is>
       </c>
     </row>
@@ -4829,7 +4829,7 @@
         </is>
       </c>
       <c r="B6" s="14" t="n">
-        <v>1200000</v>
+        <v>1560000</v>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="B7" s="14" t="n">
-        <v>3000000</v>
+        <v>3900000</v>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>

</xml_diff>